<commit_message>
Let wait-mode page delay be set in seconds, and fix Power Query M.
The Angular form and Products_AsyncWait.pq send X-Demo-Wait-Delay-Milliseconds so wait vs page delay is client-controlled (both in seconds). Rename the reserved M identifier meta to responseMeta in all three scripts.
</commit_message>
<xml_diff>
--- a/excel/OData-Query-Scenarios.xlsx
+++ b/excel/OData-Query-Scenarios.xlsx
@@ -1248,11 +1248,11 @@
                     ManualStatusHandling = {200, 202, 404, 410, 500}
                 ]
             ),
-            meta = Value.Metadata(binary)
+            responseMeta = Value.Metadata(binary)
         in
             [
-                Status = meta[Response.Status],
-                Headers = meta[Headers],
+                Status = responseMeta[Response.Status],
+                Headers = responseMeta[Headers],
                 Binary = binary
             ],
     FetchResource = (url as text) as record =&gt;
@@ -1379,11 +1379,11 @@
                     ManualStatusHandling = {200, 202, 404, 410, 500}
                 ]
             ),
-            meta = Value.Metadata(binary)
+            responseMeta = Value.Metadata(binary)
         in
             [
-                Status = meta[Response.Status],
-                Headers = meta[Headers],
+                Status = responseMeta[Response.Status],
+                Headers = responseMeta[Headers],
                 Binary = binary
             ],
     PollUntilComplete = (monitorUrl as text, attemptsLeft as number) as record =&gt;
@@ -1497,8 +1497,8 @@
 //   If the page finishes in N seconds the first response is 200 (no poll);
 //   otherwise 202 + poll Location.
 //   Continuation pages use wait=min(N, 5) — NextPageWaitSeconds — matching the web app.
-//   The service sleeps WaitQueryDelayMilliseconds (4s) on each wait-mode page, so
-//   N=2 yields 202 and N&gt;=4 yields 200. Matches the Angular default wait of 2.
+//   WaitQueryDelaySeconds matches the Angular "wait-mode page delay (seconds)" box.
+//   It is sent as X-Demo-Wait-Delay-Milliseconds (seconds × 1000). If delay &gt; wait, 202.
 // Service defaults: catalog 5000, page size 500.
 // First URL matches the web app: $count=true&amp;$orderby=Id, no $top.
 // Start the sample service first: dotnet run --project ODataLongQuery
@@ -1507,6 +1507,7 @@
     FirstUrl = BaseUrl &amp; "/odata/Products?$count=true&amp;$orderby=Id",
     FirstPageWaitSeconds = 2,
     NextPageWaitSeconds = 2,
+    WaitQueryDelaySeconds = 4,
     MaxPages = 100,
     MaxPolls = 60,
     PollDelay = #duration(0, 0, 0, 2),
@@ -1529,7 +1530,11 @@
                 if prefer = null then
                     [Accept = "application/json"]
                 else
-                    [Accept = "application/json", Prefer = prefer],
+                    [
+                        Accept = "application/json",
+                        Prefer = prefer,
+                        #"X-Demo-Wait-Delay-Milliseconds" = Number.ToText(WaitQueryDelaySeconds * 1000)
+                    ],
             binary = Web.Contents(
                 url,
                 [
@@ -1537,11 +1542,11 @@
                     ManualStatusHandling = {200, 202, 404, 410, 500}
                 ]
             ),
-            meta = Value.Metadata(binary)
+            responseMeta = Value.Metadata(binary)
         in
             [
-                Status = meta[Response.Status],
-                Headers = meta[Headers],
+                Status = responseMeta[Response.Status],
+                Headers = responseMeta[Headers],
                 Binary = binary
             ],
     PollUntilComplete = (monitorUrl as text, attemptsLeft as number) as record =&gt;

</xml_diff>